<commit_message>
feat(asset): enhance asset management with brand and model fields
- Added `brand_id` and `model` fields to asset creation and update requests in `UnitAssetController`.
- Updated asset detail views to display brand and model information.
- Improved asset detail PDF generation to include brand details.
- Enhanced validation for brand and model fields in asset forms.
- Refactored asset detail and master asset views to accommodate new fields and improve user experience.
</commit_message>
<xml_diff>
--- a/public/docs/ImportAssetMasterTemplate.xlsx
+++ b/public/docs/ImportAssetMasterTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ACER\Documents\Collage\magang\Template Exel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ACER\Documents\Collage\magang\asset_monitoring_web\public\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0E54CAC-AD0E-42D1-9823-DC0A7617EF21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16F69713-910B-4B5E-B916-973311E05678}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4440" yWindow="1248" windowWidth="17280" windowHeight="9420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Import Aset" sheetId="1" r:id="rId1"/>
@@ -26,13 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="35">
-  <si>
-    <t>Nama Brand</t>
-  </si>
-  <si>
-    <t>lenovo</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="33">
   <si>
     <t>Nama Aset</t>
   </si>
@@ -637,64 +631,57 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="49" customWidth="1"/>
+    <col min="5" max="5" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="49" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="D1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C2" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="6" t="s">
+      <c r="D2" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="7" t="s">
-        <v>1</v>
-      </c>
       <c r="E2" s="7" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="H2" s="19" t="s">
-        <v>32</v>
+        <v>31</v>
+      </c>
+      <c r="G2" s="19" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -720,7 +707,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A1" s="20" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B1" s="20"/>
       <c r="C1" s="8"/>
@@ -730,99 +717,99 @@
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="10"/>
       <c r="B2" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="E2" s="12" t="s">
         <v>13</v>
-      </c>
-      <c r="D2" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="E2" s="12" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="13"/>
       <c r="B3" s="16" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C3" s="14">
         <v>100</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E3" s="15"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B4" s="18" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C4" s="17"/>
       <c r="D4" s="17" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B5" s="18" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C5" s="17"/>
       <c r="D5" s="17" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B6" s="18" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C6" s="17"/>
       <c r="D6" s="17" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B7" s="17" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C7" s="17"/>
       <c r="D7" s="17" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E7" s="17"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B8" s="18" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C8" s="17"/>
       <c r="D8" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" s="18" t="s">
         <v>21</v>
-      </c>
-      <c r="E8" s="18" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B9" s="18" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C9" s="17"/>
       <c r="D9" s="17" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>